<commit_message>
Add clarification in sex item
</commit_message>
<xml_diff>
--- a/inst/formr/bvq-1.0.4/bvq_04_demo.xlsx
+++ b/inst/formr/bvq-1.0.4/bvq_04_demo.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="64">
   <si>
     <t xml:space="preserve">type</t>
   </si>
@@ -90,10 +90,29 @@
     <t xml:space="preserve">sex</t>
   </si>
   <si>
-    <t xml:space="preserve">### `r paste0(dplyr::case_when(bvq_01_log$language=="catalan" ~paste0("Sexe del bebé:"), bvq_01_log$language=="spanish" ~paste0("Sexo del bebé:"), TRUE ~ paste0("Sex of the baby:")))`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">left400 label_align_left answer_align_left</t>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">### `r paste0(dplyr::case_when(bvq_01_log$language=="catalan" ~paste0("Sexe del bebé"), bvq_01_log$language=="spanish" ~paste0("Sexo del bebé"), TRUE ~ paste0("Sex of the baby")))`
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">`r paste0(dplyr::case_when(bvq_01_log$language=="catalan" ~paste0("Sexe assignat al bebè en el moment del naixement"), bvq_01_log$language=="spanish" ~paste0("Sexo asignado al bebé en el momento del nacimiento"), TRUE ~ paste0("Sex assigned to the baby at birth")))`</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">answer_below_label answer_align_left</t>
   </si>
   <si>
     <t xml:space="preserve">text 5</t>
@@ -106,13 +125,10 @@
 `r paste0(dplyr::case_when(bvq_01_log$language == "catalan" ~paste0("Si us plau, indica'ns el teu codi postal:"), bvq_01_log$language == "spanish" ~paste0("Por favor, indícanos tu código postal:"), TRUE ~ paste0("Please, indicate your postcode:")))`</t>
   </si>
   <si>
-    <t xml:space="preserve">answer_below_label answer_align_left</t>
-  </si>
-  <si>
     <t xml:space="preserve">demo_parent_info</t>
   </si>
   <si>
-    <t xml:space="preserve">### `r paste0(dplyr::case_when(bvq_01_log$language == "catalan" ~paste0("Informació sobre les dues persones que més temps passen amb el/la nen/a:"), bvq_01_log$language == "spanish"~paste0("Información sobre dos personas que más tiempo pasan con el/la niño/a:"), TRUE ~ paste0("Information about the two people who spend more time with the child:")))`</t>
+    <t xml:space="preserve">## `r paste0(dplyr::case_when(bvq_01_log$language == "catalan" ~paste0("Informació sobre les dues persones que més temps passen amb el/la nen/a"), bvq_01_log$language == "spanish"~paste0("Información sobre dos personas que más tiempo pasan con el/la niño/a"), TRUE ~ paste0("Information about the two people who spend more time with the child")))`</t>
   </si>
   <si>
     <t xml:space="preserve">select_one  demo_education1</t>
@@ -185,9 +201,6 @@
   </si>
   <si>
     <t xml:space="preserve">demo_education2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`r paste0(dplyr::case_when(bvq_01_log$language == "catalan" ~paste0("Femení"), bvq_01_log$language == "spanish" ~paste0("Femenno"), TRUE ~ paste0("Female")))`</t>
   </si>
   <si>
     <t xml:space="preserve">item</t>
@@ -233,7 +246,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="16"/>
       <color rgb="FF000000"/>
@@ -263,6 +276,12 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -307,7 +326,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -326,6 +345,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -348,34 +371,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -521,7 +544,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I1048576"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="20.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="20.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="60.92"/>
@@ -529,7 +552,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="44.16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="40.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="35.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -558,7 +581,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="81" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="52.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -581,7 +604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="81" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="52.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -604,7 +627,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="81" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="52.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
@@ -627,17 +650,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="55.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="5" t="s">
         <v>22</v>
       </c>
       <c r="H5" s="1" t="s">
@@ -647,7 +670,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="344.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="138.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>23</v>
       </c>
@@ -658,7 +681,7 @@
         <v>25</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>13</v>
@@ -667,15 +690,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="263.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>28</v>
       </c>
       <c r="D7" s="1" t="n">
         <v>1</v>
@@ -687,18 +710,18 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="202.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="E8" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>13</v>
@@ -707,18 +730,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="202.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="E9" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>13</v>
@@ -727,15 +750,15 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="141.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>37</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>13</v>
@@ -762,14 +785,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C1048576"/>
-  <sheetFormatPr defaultColWidth="20" defaultRowHeight="20.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="20" defaultRowHeight="20.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -778,149 +801,139 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="182.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="1" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="182.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="C3" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C8" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="1" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="202.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B4" s="1" t="s">
+      <c r="C10" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="1" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="182.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="1" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="162" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B6" s="1" t="s">
+      <c r="C12" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="1" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="182.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="1" t="s">
+      <c r="C13" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="182.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="182.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="202.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="182.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="162" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="182.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="141.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
+    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -939,28 +952,28 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultColWidth="20" defaultRowHeight="20.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="20" defaultRowHeight="20.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="C1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="40.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>100</v>
@@ -968,15 +981,15 @@
     </row>
     <row r="4" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="40.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0</v>
@@ -984,17 +997,17 @@
     </row>
     <row r="6" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0</v>
@@ -1002,17 +1015,17 @@
     </row>
     <row r="9" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0</v>
@@ -1020,7 +1033,7 @@
     </row>
     <row r="12" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0</v>

</xml_diff>